<commit_message>
Use WMim 'intermediate' instead of WMtz annotation
</commit_message>
<xml_diff>
--- a/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k11.xlsx
+++ b/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k11.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{16F868A8-2676-6140-97ED-23A6837CD0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{428C8B0B-B93A-4446-A292-B8D9BE3E0353}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{16F868A8-2676-6140-97ED-23A6837CD0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDE88110-2AB7-7844-AA2D-2B7857BD64E8}"/>
   <bookViews>
     <workbookView xWindow="-28360" yWindow="220" windowWidth="27640" windowHeight="11900" xr2:uid="{3CAB2BDD-3107-E940-A67F-AC23A5393E98}"/>
   </bookViews>
@@ -217,10 +217,10 @@
     <t>WMuf</t>
   </si>
   <si>
-    <t>WMtz</t>
-  </si>
-  <si>
     <t>anno</t>
+  </si>
+  <si>
+    <t>WMim</t>
   </si>
 </sst>
 </file>
@@ -762,6 +762,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1110,7 +1114,7 @@
         <v>42</v>
       </c>
       <c r="G1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1340,7 +1344,7 @@
         <v>9</v>
       </c>
       <c r="G11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update annotations in vSpD k11 table
</commit_message>
<xml_diff>
--- a/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k11.xlsx
+++ b/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k11.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{16F868A8-2676-6140-97ED-23A6837CD0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDE88110-2AB7-7844-AA2D-2B7857BD64E8}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="8_{16F868A8-2676-6140-97ED-23A6837CD0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4D2EE11-C7CC-0446-8358-D9C8213CF337}"/>
   <bookViews>
-    <workbookView xWindow="-28360" yWindow="220" windowWidth="27640" windowHeight="11900" xr2:uid="{3CAB2BDD-3107-E940-A67F-AC23A5393E98}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="27600" windowHeight="17580" xr2:uid="{3CAB2BDD-3107-E940-A67F-AC23A5393E98}"/>
   </bookViews>
   <sheets>
     <sheet name="ERC_SpD_spatial_registration_an" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ERC_SpD_spatial_registration_an!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ERC_SpD_spatial_registration_an!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="87">
   <si>
     <t>cluster</t>
   </si>
@@ -163,18 +163,12 @@
     <t>L1</t>
   </si>
   <si>
-    <t>L5</t>
-  </si>
-  <si>
     <t>L6</t>
   </si>
   <si>
     <t>L2</t>
   </si>
   <si>
-    <t>L3</t>
-  </si>
-  <si>
     <t>LD</t>
   </si>
   <si>
@@ -220,7 +214,76 @@
     <t>anno</t>
   </si>
   <si>
-    <t>WMim</t>
+    <t>top_enrich_genes</t>
+  </si>
+  <si>
+    <t>sum_umi_median</t>
+  </si>
+  <si>
+    <t>sum_gene_median</t>
+  </si>
+  <si>
+    <t>expr_chrM_ratio_median</t>
+  </si>
+  <si>
+    <t>HBA1, HBA2, HBB, TAGLN, S100A6, ACTA2, IGFBP7, COL1A2, COL1A1, SLC13A4</t>
+  </si>
+  <si>
+    <t>CST3, MT1F, SLC1A3, GLUL, MT1E, MT3, TTYH1, ENHO, FBXO2, PON2</t>
+  </si>
+  <si>
+    <t>BTBD3, LAMP5, MAPK1, ATP6V1H, NCAM2, RTN4, HPCAL1, PSD3, HOPX, NCDN</t>
+  </si>
+  <si>
+    <t>SLC6A1, GAD1, DNER, GAD2, SST, CNR1, TAC1, FXYD6, NXPH1, KCNC2</t>
+  </si>
+  <si>
+    <t>COX6A1, MAP1A, COX5B, TUBB2B, ENHO, C9orf16, CCDC85B, NAA38, HOPX, NDUFA4</t>
+  </si>
+  <si>
+    <t>GPR6, RTN3, NTNG1, NECAB1, WASF1, TUBB3, COL5A2, HMGCS1, DCLK1, SERPINI1</t>
+  </si>
+  <si>
+    <t>TUBA1B, PCP4, SV2B, SSBP3, IPCEF1, SNCA, NUAK1, SYT1, HS3ST2, STMN2</t>
+  </si>
+  <si>
+    <t>DIRAS2, EFHD2, NNAT, CCN2, HS3ST4, KRT17, TBR1, NCALD, LMO3, OLFML2B</t>
+  </si>
+  <si>
+    <t>MBP, CPLX3, MOBP, AQP1, AL627171.2, KIF1C, TP53INP2, BCAS1, PAQR6, KRT17</t>
+  </si>
+  <si>
+    <t>MTURN, SNHG6, MAP4K4, PAQR6, TP53INP2, RPL21, ANKRD40, RPL37, RPS29, RPL37A</t>
+  </si>
+  <si>
+    <t>SLAIN1, ABCA2, EDIL3, DBNDD2, CNP, SIRT2, CLDND1, SLC44A1, PLLP, CBR1</t>
+  </si>
+  <si>
+    <t>median_nuclei</t>
+  </si>
+  <si>
+    <t>prop_zero_nuc</t>
+  </si>
+  <si>
+    <t>L5a</t>
+  </si>
+  <si>
+    <t>L5b</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>change from L3 (8/25)</t>
+  </si>
+  <si>
+    <t>change from LD (8/25)</t>
+  </si>
+  <si>
+    <t>change from Wmim (8/25)</t>
+  </si>
+  <si>
+    <t>Wma</t>
   </si>
 </sst>
 </file>
@@ -660,7 +723,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -703,11 +766,14 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="42" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -747,6 +813,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
     <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Percent" xfId="42" builtinId="5"/>
     <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
@@ -1085,16 +1152,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D42322D1-B7BD-1843-A441-67A7916283FA}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="17.5" customWidth="1"/>
-    <col min="3" max="3" width="44.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="55.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.1640625" customWidth="1"/>
     <col min="5" max="5" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1108,16 +1175,37 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F1" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="G1" t="s">
         <v>64</v>
       </c>
+      <c r="H1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I1" t="s">
+        <v>66</v>
+      </c>
+      <c r="J1" t="s">
+        <v>78</v>
+      </c>
+      <c r="K1" t="s">
+        <v>79</v>
+      </c>
+      <c r="L1" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" t="s">
+        <v>62</v>
+      </c>
+      <c r="N1" t="s">
+        <v>82</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1131,16 +1219,34 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F2">
+        <v>57</v>
+      </c>
+      <c r="F2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2">
+        <v>1716</v>
+      </c>
+      <c r="H2">
+        <v>898</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0.20068027210884301</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0.23006923837784399</v>
+      </c>
+      <c r="L2">
         <v>0</v>
       </c>
-      <c r="G2" t="s">
+      <c r="M2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1154,16 +1260,34 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F3">
+        <v>55</v>
+      </c>
+      <c r="F3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G3">
+        <v>2408</v>
+      </c>
+      <c r="H3">
+        <v>1019</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0.34354722422494499</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0.13364900858242099</v>
+      </c>
+      <c r="L3">
         <v>1</v>
       </c>
-      <c r="G3" t="s">
+      <c r="M3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1177,16 +1301,34 @@
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4">
+        <v>5609</v>
+      </c>
+      <c r="H4">
+        <v>2483</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0.18662581590515501</v>
+      </c>
+      <c r="J4">
+        <v>5</v>
+      </c>
+      <c r="K4" s="2">
+        <v>8.1100291420854398E-2</v>
+      </c>
+      <c r="L4">
         <v>2</v>
       </c>
-      <c r="G4" t="s">
-        <v>48</v>
+      <c r="M4" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -1200,16 +1342,34 @@
         <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5">
+        <v>5240</v>
+      </c>
+      <c r="H5">
+        <v>2370</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0.20379023883696701</v>
+      </c>
+      <c r="J5">
+        <v>6</v>
+      </c>
+      <c r="K5" s="2">
+        <v>1.4468788755684201E-2</v>
+      </c>
+      <c r="L5">
         <v>3</v>
       </c>
-      <c r="G5" t="s">
+      <c r="M5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1223,16 +1383,37 @@
         <v>17</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6">
+        <v>51</v>
+      </c>
+      <c r="F6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6">
+        <v>3920</v>
+      </c>
+      <c r="H6">
+        <v>1754</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0.25939071280686099</v>
+      </c>
+      <c r="J6">
         <v>4</v>
       </c>
-      <c r="G6" t="s">
-        <v>49</v>
+      <c r="K6" s="2">
+        <v>0.120182298992854</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6" t="s">
+        <v>48</v>
+      </c>
+      <c r="N6" t="s">
+        <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1246,16 +1427,37 @@
         <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F7">
+        <v>52</v>
+      </c>
+      <c r="F7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7">
+        <v>5851</v>
+      </c>
+      <c r="H7">
+        <v>2585</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.19890807141803099</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" s="2">
+        <v>5.2345167141746599E-2</v>
+      </c>
+      <c r="L7">
         <v>5</v>
       </c>
-      <c r="G7" t="s">
-        <v>50</v>
+      <c r="M7" t="s">
+        <v>80</v>
+      </c>
+      <c r="N7" t="s">
+        <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1269,16 +1471,34 @@
         <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F8">
+        <v>53</v>
+      </c>
+      <c r="F8" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8">
+        <v>5373.5</v>
+      </c>
+      <c r="H8">
+        <v>2420.5</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0.18848424692931001</v>
+      </c>
+      <c r="J8">
         <v>6</v>
       </c>
-      <c r="G8" t="s">
-        <v>46</v>
+      <c r="K8" s="2">
+        <v>6.3526834611172006E-2</v>
+      </c>
+      <c r="L8">
+        <v>6</v>
+      </c>
+      <c r="M8" t="s">
+        <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1292,16 +1512,34 @@
         <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9">
+        <v>3430</v>
+      </c>
+      <c r="H9">
+        <v>1643.5</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0.229469398854656</v>
+      </c>
+      <c r="J9">
+        <v>6</v>
+      </c>
+      <c r="K9" s="2">
+        <v>5.5196590596645598E-2</v>
+      </c>
+      <c r="L9">
         <v>7</v>
       </c>
-      <c r="G9" t="s">
-        <v>47</v>
+      <c r="M9" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -1315,16 +1553,34 @@
         <v>41</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
-      </c>
-      <c r="F10">
+        <v>56</v>
+      </c>
+      <c r="F10" t="s">
+        <v>75</v>
+      </c>
+      <c r="G10">
+        <v>478</v>
+      </c>
+      <c r="H10">
+        <v>285</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0.26744186046511598</v>
+      </c>
+      <c r="J10">
+        <v>7</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.109355509355509</v>
+      </c>
+      <c r="L10">
         <v>8</v>
       </c>
-      <c r="G10" t="s">
-        <v>63</v>
+      <c r="M10" t="s">
+        <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -1338,16 +1594,37 @@
         <v>37</v>
       </c>
       <c r="E11" t="s">
-        <v>61</v>
-      </c>
-      <c r="F11">
+        <v>59</v>
+      </c>
+      <c r="F11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11">
+        <v>1442.5</v>
+      </c>
+      <c r="H11">
+        <v>745</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0.233182160976278</v>
+      </c>
+      <c r="J11">
         <v>9</v>
       </c>
-      <c r="G11" t="s">
-        <v>65</v>
+      <c r="K11" s="2">
+        <v>4.84619140625E-2</v>
+      </c>
+      <c r="L11">
+        <v>9</v>
+      </c>
+      <c r="M11" t="s">
+        <v>86</v>
+      </c>
+      <c r="N11" t="s">
+        <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1361,15 +1638,34 @@
         <v>37</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
-      </c>
-      <c r="F12">
+        <v>56</v>
+      </c>
+      <c r="F12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12">
+        <v>1949</v>
+      </c>
+      <c r="H12">
+        <v>1012</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0.18453427065026301</v>
+      </c>
+      <c r="J12">
+        <v>11</v>
+      </c>
+      <c r="K12" s="2">
+        <v>1.7456853798849401E-2</v>
+      </c>
+      <c r="L12">
         <v>10</v>
       </c>
-      <c r="G12" t="s">
-        <v>62</v>
+      <c r="M12" t="s">
+        <v>60</v>
       </c>
     </row>
+    <row r="13" spans="1:14" ht="7" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update vSpD annotations and colors to WMpv
</commit_message>
<xml_diff>
--- a/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k11.xlsx
+++ b/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k11.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="8_{16F868A8-2676-6140-97ED-23A6837CD0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82B51C87-3614-1643-A0E6-B5459A4ABD63}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{16F868A8-2676-6140-97ED-23A6837CD0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5F39786-D267-E24C-83FC-22A3109AE7F5}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="21980" windowHeight="17580" xr2:uid="{3CAB2BDD-3107-E940-A67F-AC23A5393E98}"/>
   </bookViews>
@@ -280,10 +280,10 @@
     <t>change from LD (8/25)</t>
   </si>
   <si>
-    <t>change from Wmim (8/25)</t>
-  </si>
-  <si>
-    <t>WMa</t>
+    <t>WMpv</t>
+  </si>
+  <si>
+    <t>change from Wim (8/25)</t>
   </si>
 </sst>
 </file>
@@ -1618,10 +1618,10 @@
         <v>9</v>
       </c>
       <c r="M11" t="s">
+        <v>85</v>
+      </c>
+      <c r="N11" t="s">
         <v>86</v>
-      </c>
-      <c r="N11" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">

</xml_diff>